<commit_message>
Add Yerevan order template and update order template
</commit_message>
<xml_diff>
--- a/cronoi_project/cronoi_ls_siparis_sablonu.xlsx
+++ b/cronoi_project/cronoi_ls_siparis_sablonu.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3212FBF4-BD0B-421E-949D-6AF09B06AE37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8F742E9-E05D-4522-98D7-B68BF920383E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="61">
   <si>
     <t>🚛  CRONOI LS — SİPARİŞ YÜKLEME ŞABLONU</t>
   </si>
@@ -218,6 +218,9 @@
   <si>
     <t>Yükseklik
 (cm) *</t>
+  </si>
+  <si>
+    <t>vertical</t>
   </si>
 </sst>
 </file>
@@ -396,7 +399,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -419,6 +422,10 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -433,17 +440,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -808,83 +804,83 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="30.45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-      <c r="P1" s="10"/>
-      <c r="Q1" s="10"/>
-      <c r="R1" s="10"/>
-      <c r="S1" s="10"/>
-      <c r="T1" s="10"/>
-      <c r="U1" s="10"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12"/>
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
+      <c r="T1" s="12"/>
+      <c r="U1" s="12"/>
     </row>
     <row r="2" spans="1:21" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="11"/>
-      <c r="N2" s="11"/>
-      <c r="O2" s="11"/>
-      <c r="P2" s="11"/>
-      <c r="Q2" s="11"/>
-      <c r="R2" s="11"/>
-      <c r="S2" s="11"/>
-      <c r="T2" s="11"/>
-      <c r="U2" s="11"/>
+      <c r="A2" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="13"/>
+      <c r="T2" s="13"/>
+      <c r="U2" s="13"/>
     </row>
     <row r="3" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="13" t="s">
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
-      <c r="M3" s="13"/>
-      <c r="N3" s="14" t="s">
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15"/>
+      <c r="N3" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="O3" s="14"/>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
-      <c r="R3" s="14"/>
-      <c r="S3" s="14"/>
-      <c r="T3" s="14"/>
-      <c r="U3" s="14"/>
+      <c r="O3" s="16"/>
+      <c r="P3" s="16"/>
+      <c r="Q3" s="16"/>
+      <c r="R3" s="16"/>
+      <c r="S3" s="16"/>
+      <c r="T3" s="16"/>
+      <c r="U3" s="16"/>
     </row>
     <row r="4" spans="1:21" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -935,13 +931,13 @@
       <c r="P4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="Q4" s="18" t="s">
+      <c r="Q4" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="R4" s="18" t="s">
+      <c r="R4" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="S4" s="18" t="s">
+      <c r="S4" s="3" t="s">
         <v>59</v>
       </c>
       <c r="T4" s="3" t="s">
@@ -982,7 +978,7 @@
       <c r="J5" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K5" s="15" t="s">
+      <c r="K5" t="s">
         <v>28</v>
       </c>
       <c r="L5" s="5" t="s">
@@ -991,28 +987,30 @@
       <c r="M5" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="N5" s="16" t="s">
+      <c r="N5" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="O5" s="17" t="s">
+      <c r="O5" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="P5" s="16">
+      <c r="P5" s="10">
         <v>32</v>
       </c>
-      <c r="Q5" s="16">
+      <c r="Q5" s="10">
         <v>185</v>
       </c>
-      <c r="R5" s="16">
+      <c r="R5" s="10">
         <v>15</v>
       </c>
-      <c r="S5" s="16">
+      <c r="S5" s="10">
         <v>105</v>
       </c>
       <c r="T5" s="6">
         <v>1</v>
       </c>
-      <c r="U5" s="6"/>
+      <c r="U5" s="6" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="6" spans="1:21" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
@@ -1045,37 +1043,39 @@
       <c r="J6" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K6" s="15" t="s">
+      <c r="K6" t="s">
         <v>28</v>
       </c>
       <c r="L6" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M6" s="19" t="s">
+      <c r="M6" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="N6" s="16" t="s">
+      <c r="N6" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="O6" s="17" t="s">
+      <c r="O6" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="P6" s="16">
+      <c r="P6" s="10">
         <v>4</v>
       </c>
-      <c r="Q6" s="16">
+      <c r="Q6" s="10">
         <v>165</v>
       </c>
-      <c r="R6" s="16">
+      <c r="R6" s="10">
         <v>15</v>
       </c>
-      <c r="S6" s="16">
+      <c r="S6" s="10">
         <v>105</v>
       </c>
       <c r="T6" s="6">
         <v>1</v>
       </c>
-      <c r="U6" s="6"/>
+      <c r="U6" s="6" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="7" spans="1:21" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
@@ -1108,37 +1108,39 @@
       <c r="J7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K7" s="15" t="s">
+      <c r="K7" t="s">
         <v>28</v>
       </c>
       <c r="L7" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M7" s="19" t="s">
+      <c r="M7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="N7" s="16" t="s">
+      <c r="N7" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="O7" s="17" t="s">
+      <c r="O7" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="P7" s="16">
+      <c r="P7" s="10">
         <v>60</v>
       </c>
-      <c r="Q7" s="16">
+      <c r="Q7" s="10">
         <v>155</v>
       </c>
-      <c r="R7" s="16">
+      <c r="R7" s="10">
         <v>15</v>
       </c>
-      <c r="S7" s="16">
+      <c r="S7" s="10">
         <v>105</v>
       </c>
       <c r="T7" s="6">
         <v>1</v>
       </c>
-      <c r="U7" s="6"/>
+      <c r="U7" s="6" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="8" spans="1:21" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
@@ -1171,37 +1173,39 @@
       <c r="J8" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K8" s="15" t="s">
+      <c r="K8" t="s">
         <v>28</v>
       </c>
       <c r="L8" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M8" s="19" t="s">
+      <c r="M8" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="N8" s="16" t="s">
+      <c r="N8" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="O8" s="17" t="s">
+      <c r="O8" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="P8" s="16">
+      <c r="P8" s="10">
         <v>36</v>
       </c>
-      <c r="Q8" s="16">
+      <c r="Q8" s="10">
         <v>105</v>
       </c>
-      <c r="R8" s="16">
+      <c r="R8" s="10">
         <v>15</v>
       </c>
-      <c r="S8" s="16">
+      <c r="S8" s="10">
         <v>105</v>
       </c>
       <c r="T8" s="6">
         <v>1</v>
       </c>
-      <c r="U8" s="6"/>
+      <c r="U8" s="6" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
@@ -1234,37 +1238,39 @@
       <c r="J9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K9" s="15" t="s">
+      <c r="K9" t="s">
         <v>28</v>
       </c>
       <c r="L9" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M9" s="19" t="s">
+      <c r="M9" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="N9" s="16" t="s">
+      <c r="N9" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="O9" s="17" t="s">
+      <c r="O9" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="P9" s="16">
+      <c r="P9" s="10">
         <v>2</v>
       </c>
-      <c r="Q9" s="16">
+      <c r="Q9" s="10">
         <v>195</v>
       </c>
-      <c r="R9" s="16">
+      <c r="R9" s="10">
         <v>15</v>
       </c>
-      <c r="S9" s="16">
+      <c r="S9" s="10">
         <v>105</v>
       </c>
       <c r="T9" s="6">
         <v>1</v>
       </c>
-      <c r="U9" s="6"/>
+      <c r="U9" s="6" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
@@ -1297,31 +1303,31 @@
       <c r="J10" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K10" s="15" t="s">
+      <c r="K10" t="s">
         <v>28</v>
       </c>
       <c r="L10" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M10" s="19" t="s">
+      <c r="M10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="N10" s="16" t="s">
+      <c r="N10" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="O10" s="17" t="s">
+      <c r="O10" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="P10" s="16">
+      <c r="P10" s="10">
         <v>61</v>
       </c>
-      <c r="Q10" s="16">
+      <c r="Q10" s="10">
         <v>80</v>
       </c>
-      <c r="R10" s="16">
+      <c r="R10" s="10">
         <v>85</v>
       </c>
-      <c r="S10" s="16">
+      <c r="S10" s="10">
         <v>95</v>
       </c>
       <c r="T10" s="6">
@@ -1360,31 +1366,31 @@
       <c r="J11" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K11" s="15" t="s">
+      <c r="K11" t="s">
         <v>28</v>
       </c>
       <c r="L11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M11" s="19" t="s">
+      <c r="M11" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="N11" s="16" t="s">
+      <c r="N11" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="O11" s="17" t="s">
+      <c r="O11" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="P11" s="16">
+      <c r="P11" s="10">
         <v>13</v>
       </c>
-      <c r="Q11" s="16">
+      <c r="Q11" s="10">
         <v>80</v>
       </c>
-      <c r="R11" s="16">
+      <c r="R11" s="10">
         <v>85</v>
       </c>
-      <c r="S11" s="16">
+      <c r="S11" s="10">
         <v>95</v>
       </c>
       <c r="T11" s="6">
@@ -1423,31 +1429,31 @@
       <c r="J12" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K12" s="15" t="s">
+      <c r="K12" t="s">
         <v>28</v>
       </c>
       <c r="L12" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M12" s="19" t="s">
+      <c r="M12" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="N12" s="16" t="s">
+      <c r="N12" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="O12" s="17" t="s">
+      <c r="O12" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="P12" s="16">
+      <c r="P12" s="10">
         <v>38</v>
       </c>
-      <c r="Q12" s="16">
+      <c r="Q12" s="10">
         <v>80</v>
       </c>
-      <c r="R12" s="16">
+      <c r="R12" s="10">
         <v>85</v>
       </c>
-      <c r="S12" s="16">
+      <c r="S12" s="10">
         <v>95</v>
       </c>
       <c r="T12" s="6">
@@ -1486,31 +1492,31 @@
       <c r="J13" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K13" s="15" t="s">
+      <c r="K13" t="s">
         <v>28</v>
       </c>
       <c r="L13" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M13" s="19" t="s">
+      <c r="M13" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="N13" s="16" t="s">
+      <c r="N13" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="O13" s="17" t="s">
+      <c r="O13" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="P13" s="16">
+      <c r="P13" s="10">
         <v>2</v>
       </c>
-      <c r="Q13" s="16">
+      <c r="Q13" s="10">
         <v>80</v>
       </c>
-      <c r="R13" s="16">
+      <c r="R13" s="10">
         <v>85</v>
       </c>
-      <c r="S13" s="16">
+      <c r="S13" s="10">
         <v>95</v>
       </c>
       <c r="T13" s="6">
@@ -1549,31 +1555,31 @@
       <c r="J14" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K14" s="15" t="s">
+      <c r="K14" t="s">
         <v>28</v>
       </c>
       <c r="L14" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M14" s="19" t="s">
+      <c r="M14" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="N14" s="16" t="s">
+      <c r="N14" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="O14" s="17" t="s">
+      <c r="O14" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="P14" s="16">
+      <c r="P14" s="10">
         <v>84</v>
       </c>
-      <c r="Q14" s="16">
+      <c r="Q14" s="10">
         <v>50</v>
       </c>
-      <c r="R14" s="16">
+      <c r="R14" s="10">
         <v>60</v>
       </c>
-      <c r="S14" s="16">
+      <c r="S14" s="10">
         <v>85</v>
       </c>
       <c r="T14" s="6">
@@ -1612,31 +1618,31 @@
       <c r="J15" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K15" s="15" t="s">
+      <c r="K15" t="s">
         <v>28</v>
       </c>
       <c r="L15" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M15" s="19" t="s">
+      <c r="M15" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="N15" s="16" t="s">
+      <c r="N15" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="O15" s="17" t="s">
+      <c r="O15" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="P15" s="16">
+      <c r="P15" s="10">
         <v>2</v>
       </c>
-      <c r="Q15" s="16">
+      <c r="Q15" s="10">
         <v>50</v>
       </c>
-      <c r="R15" s="16">
+      <c r="R15" s="10">
         <v>60</v>
       </c>
-      <c r="S15" s="16">
+      <c r="S15" s="10">
         <v>85</v>
       </c>
       <c r="T15" s="6">
@@ -1675,31 +1681,31 @@
       <c r="J16" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K16" s="15" t="s">
+      <c r="K16" t="s">
         <v>28</v>
       </c>
       <c r="L16" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M16" s="19" t="s">
+      <c r="M16" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="N16" s="16" t="s">
+      <c r="N16" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="O16" s="17" t="s">
+      <c r="O16" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="P16" s="16">
+      <c r="P16" s="10">
         <v>80</v>
       </c>
-      <c r="Q16" s="16">
+      <c r="Q16" s="10">
         <v>75</v>
       </c>
-      <c r="R16" s="16">
+      <c r="R16" s="10">
         <v>75</v>
       </c>
-      <c r="S16" s="16">
+      <c r="S16" s="10">
         <v>70</v>
       </c>
       <c r="T16" s="6">
@@ -1718,7 +1724,6 @@
       <c r="H17" s="7"/>
       <c r="I17" s="8"/>
       <c r="J17" s="8"/>
-      <c r="K17" s="15"/>
       <c r="L17" s="5"/>
       <c r="M17" s="5"/>
       <c r="N17" s="9"/>
@@ -1741,7 +1746,6 @@
       <c r="H18" s="7"/>
       <c r="I18" s="8"/>
       <c r="J18" s="8"/>
-      <c r="K18" s="15"/>
       <c r="L18" s="5"/>
       <c r="M18" s="5"/>
       <c r="N18" s="9"/>
@@ -1764,7 +1768,6 @@
       <c r="H19" s="7"/>
       <c r="I19" s="8"/>
       <c r="J19" s="8"/>
-      <c r="K19" s="15"/>
       <c r="L19" s="5"/>
       <c r="M19" s="5"/>
       <c r="N19" s="9"/>
@@ -1787,7 +1790,6 @@
       <c r="H20" s="7"/>
       <c r="I20" s="8"/>
       <c r="J20" s="8"/>
-      <c r="K20" s="15"/>
       <c r="L20" s="5"/>
       <c r="M20" s="5"/>
       <c r="N20" s="9"/>
@@ -1810,7 +1812,6 @@
       <c r="H21" s="7"/>
       <c r="I21" s="8"/>
       <c r="J21" s="8"/>
-      <c r="K21" s="15"/>
       <c r="L21" s="5"/>
       <c r="M21" s="5"/>
       <c r="N21" s="9"/>
@@ -1833,7 +1834,6 @@
       <c r="H22" s="7"/>
       <c r="I22" s="8"/>
       <c r="J22" s="8"/>
-      <c r="K22" s="15"/>
       <c r="L22" s="5"/>
       <c r="M22" s="5"/>
       <c r="N22" s="9"/>
@@ -1856,7 +1856,6 @@
       <c r="H23" s="7"/>
       <c r="I23" s="8"/>
       <c r="J23" s="8"/>
-      <c r="K23" s="15"/>
       <c r="L23" s="5"/>
       <c r="M23" s="5"/>
       <c r="N23" s="9"/>
@@ -1879,7 +1878,6 @@
       <c r="H24" s="7"/>
       <c r="I24" s="8"/>
       <c r="J24" s="8"/>
-      <c r="K24" s="15"/>
       <c r="L24" s="5"/>
       <c r="M24" s="5"/>
       <c r="N24" s="9"/>

</xml_diff>

<commit_message>
19.06.2026 New version Lojistics
</commit_message>
<xml_diff>
--- a/cronoi_project/cronoi_ls_siparis_sablonu.xlsx
+++ b/cronoi_project/cronoi_ls_siparis_sablonu.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A92E26-3798-4D96-AC17-383F7DFA928D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02F9353E-BDC7-43D3-83E7-13823EDAB021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Siparişler" sheetId="1" r:id="rId1"/>
@@ -118,9 +118,6 @@
     <t>2026-04-02</t>
   </si>
   <si>
-    <t>O2-12714</t>
-  </si>
-  <si>
     <t>1 Amiryan St, Yerevan 0010, Ermenistan</t>
   </si>
   <si>
@@ -221,6 +218,9 @@
   </si>
   <si>
     <t>vertical</t>
+  </si>
+  <si>
+    <t>O2-12714-OPT001</t>
   </si>
 </sst>
 </file>
@@ -932,13 +932,13 @@
         <v>20</v>
       </c>
       <c r="Q4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="R4" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="R4" s="3" t="s">
+      <c r="S4" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="S4" s="3" t="s">
-        <v>59</v>
       </c>
       <c r="T4" s="3" t="s">
         <v>21</v>
@@ -949,7 +949,7 @@
     </row>
     <row r="5" spans="1:21" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="B5" s="5">
         <v>12714</v>
@@ -967,31 +967,31 @@
         <v>1</v>
       </c>
       <c r="G5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="I5" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="J5" s="5" t="s">
         <v>24</v>
       </c>
       <c r="K5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L5" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="L5" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="M5" s="5" t="s">
         <v>25</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="O5" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="P5" s="10">
         <v>32</v>
@@ -1009,12 +1009,12 @@
         <v>1</v>
       </c>
       <c r="U5" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:21" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="B6" s="5">
         <v>12714</v>
@@ -1032,31 +1032,31 @@
         <v>1</v>
       </c>
       <c r="G6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="I6" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>24</v>
       </c>
       <c r="K6" t="s">
+        <v>27</v>
+      </c>
+      <c r="L6" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="M6" s="5" t="s">
         <v>25</v>
       </c>
       <c r="N6" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="O6" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="P6" s="10">
         <v>4</v>
@@ -1074,12 +1074,12 @@
         <v>1</v>
       </c>
       <c r="U6" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:21" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="B7" s="5">
         <v>12714</v>
@@ -1097,31 +1097,31 @@
         <v>1</v>
       </c>
       <c r="G7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="I7" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="J7" s="5" t="s">
         <v>24</v>
       </c>
       <c r="K7" t="s">
+        <v>27</v>
+      </c>
+      <c r="L7" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="L7" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="M7" s="5" t="s">
         <v>25</v>
       </c>
       <c r="N7" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="O7" s="11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="P7" s="10">
         <v>60</v>
@@ -1139,12 +1139,12 @@
         <v>1</v>
       </c>
       <c r="U7" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:21" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="B8" s="5">
         <v>12714</v>
@@ -1162,31 +1162,31 @@
         <v>1</v>
       </c>
       <c r="G8" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H8" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="I8" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>24</v>
       </c>
       <c r="K8" t="s">
+        <v>27</v>
+      </c>
+      <c r="L8" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="L8" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="M8" s="5" t="s">
         <v>25</v>
       </c>
       <c r="N8" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O8" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P8" s="10">
         <v>36</v>
@@ -1204,12 +1204,12 @@
         <v>1</v>
       </c>
       <c r="U8" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="B9" s="5">
         <v>12714</v>
@@ -1227,31 +1227,31 @@
         <v>1</v>
       </c>
       <c r="G9" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="I9" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="J9" s="5" t="s">
         <v>24</v>
       </c>
       <c r="K9" t="s">
+        <v>27</v>
+      </c>
+      <c r="L9" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="L9" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="M9" s="5" t="s">
         <v>25</v>
       </c>
       <c r="N9" s="10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O9" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="P9" s="10">
         <v>2</v>
@@ -1269,12 +1269,12 @@
         <v>1</v>
       </c>
       <c r="U9" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="B10" s="5">
         <v>12714</v>
@@ -1292,31 +1292,31 @@
         <v>1</v>
       </c>
       <c r="G10" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="I10" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="J10" s="5" t="s">
         <v>24</v>
       </c>
       <c r="K10" t="s">
+        <v>27</v>
+      </c>
+      <c r="L10" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="L10" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="M10" s="5" t="s">
         <v>25</v>
       </c>
       <c r="N10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O10" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="P10" s="10">
         <v>61</v>
@@ -1337,7 +1337,7 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="B11" s="5">
         <v>12714</v>
@@ -1355,31 +1355,31 @@
         <v>1</v>
       </c>
       <c r="G11" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H11" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="I11" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="J11" s="5" t="s">
         <v>24</v>
       </c>
       <c r="K11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L11" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="L11" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="M11" s="5" t="s">
         <v>25</v>
       </c>
       <c r="N11" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="O11" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="P11" s="10">
         <v>13</v>
@@ -1400,7 +1400,7 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="B12" s="5">
         <v>12714</v>
@@ -1418,31 +1418,31 @@
         <v>1</v>
       </c>
       <c r="G12" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H12" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="I12" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="J12" s="5" t="s">
         <v>24</v>
       </c>
       <c r="K12" t="s">
+        <v>27</v>
+      </c>
+      <c r="L12" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="L12" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="M12" s="5" t="s">
         <v>25</v>
       </c>
       <c r="N12" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="O12" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="P12" s="10">
         <v>38</v>
@@ -1463,7 +1463,7 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="B13" s="5">
         <v>12714</v>
@@ -1481,31 +1481,31 @@
         <v>1</v>
       </c>
       <c r="G13" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H13" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="4" t="s">
+      <c r="I13" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="I13" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="J13" s="5" t="s">
         <v>24</v>
       </c>
       <c r="K13" t="s">
+        <v>27</v>
+      </c>
+      <c r="L13" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="L13" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="M13" s="5" t="s">
         <v>25</v>
       </c>
       <c r="N13" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="O13" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="P13" s="10">
         <v>2</v>
@@ -1526,7 +1526,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="B14" s="5">
         <v>12714</v>
@@ -1544,31 +1544,31 @@
         <v>1</v>
       </c>
       <c r="G14" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H14" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="I14" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="I14" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="J14" s="5" t="s">
         <v>24</v>
       </c>
       <c r="K14" t="s">
+        <v>27</v>
+      </c>
+      <c r="L14" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="L14" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="M14" s="5" t="s">
         <v>25</v>
       </c>
       <c r="N14" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="O14" s="11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="P14" s="10">
         <v>84</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="B15" s="5">
         <v>12714</v>
@@ -1607,31 +1607,31 @@
         <v>1</v>
       </c>
       <c r="G15" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H15" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="4" t="s">
+      <c r="I15" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="J15" s="5" t="s">
         <v>24</v>
       </c>
       <c r="K15" t="s">
+        <v>27</v>
+      </c>
+      <c r="L15" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="L15" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="M15" s="5" t="s">
         <v>25</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O15" s="11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="P15" s="10">
         <v>2</v>
@@ -1652,7 +1652,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="B16" s="5">
         <v>12714</v>
@@ -1670,31 +1670,31 @@
         <v>1</v>
       </c>
       <c r="G16" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H16" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="I16" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="I16" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="J16" s="5" t="s">
         <v>24</v>
       </c>
       <c r="K16" t="s">
+        <v>27</v>
+      </c>
+      <c r="L16" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="L16" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="M16" s="5" t="s">
         <v>25</v>
       </c>
       <c r="N16" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="O16" s="11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="P16" s="10">
         <v>80</v>

</xml_diff>